<commit_message>
Audio bus refactor, overcharged class fix, animation fallback for backgrounded tabs
</commit_message>
<xml_diff>
--- a/proto-01-line-battle/config/avui-config.xlsx
+++ b/proto-01-line-battle/config/avui-config.xlsx
@@ -819,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1128,283 +1128,328 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>layerEase</t>
+          <t>musicFadeMs</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>0.16</v>
+        <v>900</v>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>How fast layers slide to their new slot. Higher = snappier.</t>
+          <t>How quickly the theme fades out when the battle ends.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>layerWaveDelay</t>
+          <t>musicVolume</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Phase offset per slot, so breathing travels outward in waves.</t>
+          <t>Theme level. Lower this if the sound effects are getting buried.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>layerInnerShrink</t>
+          <t>sfxVolume</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>0.85</v>
+        <v>1.05</v>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Curve of the radius falloff toward the centre.</t>
+          <t>Sound-effect level, mixed against musicVolume.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>layerFill</t>
+          <t>layerEase</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>0.42</v>
+        <v>0.16</v>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Ring thickness as a fraction of the gap to the next slot.</t>
+          <t>How fast layers slide to their new slot. Higher = snappier.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>layerOuterThick</t>
+          <t>layerWaveDelay</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>2</v>
+        <v>0.85</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Thickness multiplier for the outermost (active) layer.</t>
+          <t>Phase offset per slot, so breathing travels outward in waves.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>layerInnerThick</t>
+          <t>layerInnerShrink</t>
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Thickness multiplier for every layer behind it.</t>
+          <t>Curve of the radius falloff toward the centre.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>layerFlashMs</t>
+          <t>layerFill</t>
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>240</v>
+        <v>0.42</v>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>How long a struck layer flashes white before vanishing.</t>
+          <t>Ring thickness as a fraction of the gap to the next slot.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>layerGapMs</t>
+          <t>layerOuterThick</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>260</v>
+        <v>2</v>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Beat between the layer vanishing and it regrowing at the back.</t>
+          <t>Thickness multiplier for the outermost (active) layer.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>layerRegrowMs</t>
+          <t>layerInnerThick</t>
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>380</v>
+        <v>0.9</v>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>How long the regrow beat holds before resolution continues.</t>
+          <t>Thickness multiplier for every layer behind it.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>enemyRingBaseR</t>
+          <t>layerFlashMs</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>28</v>
+        <v>240</v>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Enemy: radius of the outermost ring, in logical canvas pixels.</t>
+          <t>How long a struck layer flashes white before vanishing.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>enemyRingSpacing</t>
+          <t>layerGapMs</t>
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>4.7</v>
+        <v>260</v>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Enemy: radius step between one layer and the next in. baseR/spacing sets how many fit.</t>
+          <t>Beat between the layer vanishing and it regrowing at the back.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>enemyRingBreathe</t>
+          <t>layerRegrowMs</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>1.6</v>
+        <v>380</v>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Enemy ring breathing amplitude.</t>
+          <t>How long the regrow beat holds before resolution continues.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>playerRingBaseR</t>
+          <t>enemyRingBaseR</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>300</v>
+        <v>28</v>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Player: radius of the outermost ring. Huge on purpose — a big circle reads as a nearly flat band.</t>
+          <t>Enemy: radius of the outermost ring, in logical canvas pixels.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>playerRingSpacing</t>
+          <t>enemyRingSpacing</t>
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Player: radius step between layers. Small, so all six sit in a thin arc despite the huge radius.</t>
+          <t>Enemy: radius step between one layer and the next in. baseR/spacing sets how many fit.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>playerRingBreathe</t>
+          <t>enemyRingBreathe</t>
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Player ring breathing amplitude.</t>
+          <t>Enemy ring breathing amplitude.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>playerCanvasW</t>
+          <t>playerRingBaseR</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Player ring canvas width in logical pixels (wide and short).</t>
+          <t>Player: radius of the outermost ring. Huge on purpose — a big circle reads as a nearly flat band.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>playerCanvasH</t>
+          <t>playerRingSpacing</t>
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Player ring canvas height in logical pixels.</t>
+          <t>Player: radius step between layers. Small, so all six sit in a thin arc despite the huge radius.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>playerRingCy</t>
+          <t>playerRingBreathe</t>
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>300</v>
+        <v>2.2</v>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Player: circle centre Y, pushed far below the strip so only the flat top of the arc shows.</t>
+          <t>Player ring breathing amplitude.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
+          <t>playerCanvasW</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Player ring canvas width in logical pixels (wide and short).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>playerCanvasH</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Player ring canvas height in logical pixels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>playerRingCy</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Player: circle centre Y, pushed far below the strip so only the flat top of the arc shows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
           <t>crusherSteps</t>
         </is>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B43" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>Audio bit-crusher quantisation. Low = Atari harsh, high = SNES-clean.</t>
         </is>
@@ -1540,19 +1585,19 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>440</v>
+        <v>980</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>660</v>
+        <v>1460</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.2</v>
+        <v>0.46</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
@@ -1572,19 +1617,19 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>330</v>
+        <v>520</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.16</v>
+        <v>0.34</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.18</v>
+        <v>0.24</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Major refactor: split monolith into modular src/, styles/, config/csv/ — tap bug fix, charge bar redesign, ability shots, 3-slot line
</commit_message>
<xml_diff>
--- a/proto-01-line-battle/config/avui-config.xlsx
+++ b/proto-01-line-battle/config/avui-config.xlsx
@@ -819,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -875,11 +875,11 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Line segments per line. A charge segment consumes one, same as a station.</t>
+          <t>FALLBACK line size, used only if a unit row leaves line_cap blank.</t>
         </is>
       </c>
     </row>
@@ -1128,328 +1128,808 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>musicFadeMs</t>
+          <t>aiChargeBias</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>900</v>
+        <v>0.55</v>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>How quickly the theme fades out when the battle ends.</t>
+          <t>Chance the AI prefers an ability with charge segments when it can afford one.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>musicVolume</t>
+          <t>shuffleLayersEachRound</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Theme level. Lower this if the sound effects are getting buried.</t>
+          <t>Re-order every unit's layer queue at the start of each round.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>sfxVolume</t>
+          <t>chargeGrantsSlots</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Sound-effect level, mixed against musicVolume.</t>
+          <t>Each charge segment in a line grants the OPPONENT one temporary slot next turn.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>layerEase</t>
+          <t>maxBonusSlots</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>0.16</v>
+        <v>6</v>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>How fast layers slide to their new slot. Higher = snappier.</t>
+          <t>FALLBACK cap on temporary slots, used only if a unit row leaves max_bonus_slots blank.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>layerWaveDelay</t>
+          <t>abilPageSize</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>0.85</v>
+        <v>4</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Phase offset per slot, so breathing travels outward in waves.</t>
+          <t>Abilities shown per page in the Emotions panel.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>layerInnerShrink</t>
+          <t>slotArriveMs</t>
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>0.85</v>
+        <v>260</v>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Curve of the radius falloff toward the centre.</t>
+          <t>Gap between one temporary slot flying in and the next.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>layerFill</t>
+          <t>swipeMinPx</t>
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>0.42</v>
+        <v>36</v>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Ring thickness as a fraction of the gap to the next slot.</t>
+          <t>How far a pointer must travel across the panel to count as a page swipe.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>layerOuterThick</t>
+          <t>tagGrowth</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>2</v>
+        <v>0.85</v>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Thickness multiplier for the outermost (active) layer.</t>
+          <t>How much an accumulating tag grows once it holds a full max-MS worth of change.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>layerInnerThick</t>
+          <t>tagBreathSlowMs</t>
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>0.9</v>
+        <v>1700</v>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Thickness multiplier for every layer behind it.</t>
+          <t>Breathing period of an accumulating tag holding almost nothing.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>layerFlashMs</t>
+          <t>tagBreathFastMs</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>240</v>
+        <v>380</v>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>How long a struck layer flashes white before vanishing.</t>
+          <t>Breathing period of a tag holding a full max-MS worth — it flashes far harder.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>layerGapMs</t>
+          <t>gaugeW</t>
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>260</v>
+        <v>134</v>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Beat between the layer vanishing and it regrowing at the back.</t>
+          <t>Gauge canvas width in logical pixels. Lower = chunkier pixels, coarser value steps.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>layerRegrowMs</t>
+          <t>gaugeH</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>380</v>
+        <v>22</v>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>How long the regrow beat holds before resolution continues.</t>
+          <t>Gauge canvas height in logical pixels — tall enough for the end caps.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>enemyRingBaseR</t>
+          <t>barCoreH</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Enemy: radius of the outermost ring, in logical canvas pixels.</t>
+          <t>Height of the bar's interior, before the wave, in logical pixels.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>enemyRingSpacing</t>
+          <t>barWaveAmp</t>
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>4.7</v>
+        <v>1.4</v>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Enemy: radius step between one layer and the next in. baseR/spacing sets how many fit.</t>
+          <t>Wave amplitude on the bar's silhouette (reference: 9.8 of a 1026-long bar).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>enemyRingBreathe</t>
+          <t>barWaveHalf</t>
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>1.6</v>
+        <v>5.6</v>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Enemy ring breathing amplitude.</t>
+          <t>Half-period of the silhouette wave, i.e. one arc (reference: 43.3).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>playerRingBaseR</t>
+          <t>barWaveSpeed</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>300</v>
+        <v>0.1</v>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Player: radius of the outermost ring. Huge on purpose — a big circle reads as a nearly flat band.</t>
+          <t>How fast the silhouette wave travels.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>playerRingSpacing</t>
+          <t>ecBandFrac</t>
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>5</v>
+        <v>0.82</v>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Player: radius step between layers. Small, so all six sit in a thin arc despite the huge radius.</t>
+          <t>Charge fill height as a fraction of the bar interior (reference: 76 of 92.74).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>playerRingBreathe</t>
+          <t>ecWaveAmp</t>
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>2.2</v>
+        <v>0.7</v>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Player ring breathing amplitude.</t>
+          <t>Amplitude of the charge fill's own wave — long and shallow, per the reference.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>playerCanvasW</t>
+          <t>ecWaveHalf</t>
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>120</v>
+        <v>19</v>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Player ring canvas width in logical pixels (wide and short).</t>
+          <t>Half-period of the charge fill's wave. Much longer than the silhouette's.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>playerCanvasH</t>
+          <t>ecWaveSpeed</t>
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>32</v>
+        <v>0.05</v>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Player ring canvas height in logical pixels.</t>
+          <t>How fast the charge wave travels.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>playerRingCy</t>
+          <t>ecInnerFrac</t>
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>300</v>
+        <v>0.5</v>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Player: circle centre Y, pushed far below the strip so only the flat top of the arc shows.</t>
+          <t>Inner charge bar thickness, as a fraction of the outer one. Same shape, dodged over it.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
+          <t>ecInnerAmt</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>How hard the inner charge bar dodges. 1 blows out to white; lower keeps the hue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>arcSpacing</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Spacing of the background arc texture (reference: 23.83).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>arcRadius</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Radius of the background arcs (reference: 96.95).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>arcAlpha</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>How strongly the arcs show. They only read against the unlit stretch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>capW</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>End-cap width in logical pixels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>capR</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>End-cap corner rounding in logical pixels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>ballFlyMs</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="n">
+        <v>330</v>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>How long a ball of light takes to arc from its indicator into the bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>settleStepMs</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Pause between one hit landing on a bar and the next setting off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>barTweenMs</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>How long a bar takes to travel to its new value once a hit lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>overloadHoldMs</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>How long the OVERLOAD tag and its slow motion last.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>ecScrollSpeed</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>How fast the charge gradient drifts along the bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>musicFadeMs</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="n">
+        <v>900</v>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>How quickly the theme fades out when the battle ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>musicVolume</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Theme level. Lower this if the sound effects are getting buried.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>sfxVolume</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Sound-effect level, mixed against musicVolume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>layerEase</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>How fast layers slide to their new slot. Higher = snappier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>layerWaveDelay</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Phase offset per slot, so breathing travels outward in waves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>layerInnerShrink</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Curve of the radius falloff toward the centre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>layerFill</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Ring thickness as a fraction of the gap to the next slot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>layerOuterThick</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Thickness multiplier for the outermost (active) layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>layerInnerThick</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Thickness multiplier for every layer behind it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>layerFlashMs</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="n">
+        <v>240</v>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>How long a struck layer flashes white before vanishing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>layerGapMs</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Beat between the layer vanishing and it regrowing at the back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>layerRegrowMs</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>How long the regrow beat holds before resolution continues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>enemyRingBaseR</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>Enemy: radius of the outermost ring, in logical canvas pixels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>enemyRingSpacing</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Enemy: radius step between one layer and the next in. baseR/spacing sets how many fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>enemyRingBreathe</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>Enemy ring breathing amplitude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>playerRingBaseR</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Player: radius of the outermost ring. Huge on purpose — a big circle reads as a nearly flat band.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>playerRingSpacing</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Player: radius step between layers. Small, so all six sit in a thin arc despite the huge radius.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>playerRingBreathe</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Player ring breathing amplitude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>playerCanvasW</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Player ring canvas width in logical pixels (wide and short).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>playerCanvasH</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Player ring canvas height in logical pixels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>playerRingCy</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Player: circle centre Y, pushed far below the strip so only the flat top of the arc shows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
           <t>crusherSteps</t>
         </is>
       </c>
-      <c r="B43" s="8" t="n">
+      <c r="B75" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>Audio bit-crusher quantisation. Low = Atari harsh, high = SNES-clean.</t>
         </is>
@@ -1469,7 +1949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1608,7 +2088,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>remove</t>
+          <t>place</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1617,62 +2097,62 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>520</v>
+        <v>620</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>220</v>
+        <v>1760</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.24</v>
+        <v>0.35</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Removing a station.</t>
+          <t>The station lands on your line and flashes white.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>depart</t>
+          <t>slot</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>sawtooth</t>
+          <t>triangle</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>70</v>
+        <v>1500</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>420</v>
+        <v>150</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>0.45</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>The line departs and charge is spent.</t>
+          <t>A temporary slot flies in from the opponent.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>travel</t>
+          <t>remove</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -1681,94 +2161,94 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>150</v>
+        <v>520</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>150</v>
+        <v>220</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.1</v>
+        <v>0.34</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Line scrolling to the next station.</t>
+          <t>Removing a station.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>arrive</t>
+          <t>depart</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>square</t>
+          <t>sawtooth</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>880</v>
+        <v>240</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>880</v>
+        <v>70</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>45</v>
+        <v>420</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.14</v>
+        <v>0.26</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Station reaches the head and lights up.</t>
+          <t>The line departs and charge is spent.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>travel</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>square</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>700</v>
+        <v>150</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>700</v>
+        <v>150</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>190</v>
+        <v>38</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.34</v>
+        <v>0.1</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Off-type hit.</t>
+          <t>Line scrolling to the next station.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>absorb</t>
+          <t>arrive</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -1777,30 +2257,30 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>300</v>
+        <v>880</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1200</v>
+        <v>880</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>260</v>
+        <v>45</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>0.24</v>
+        <v>0.14</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>Same-type hit: the layer absorbs it.</t>
+          <t>Station reaches the head and lights up.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>block</t>
+          <t>hit</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -1809,213 +2289,277 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>1600</v>
+        <v>700</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1600</v>
+        <v>700</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>90</v>
+        <v>190</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Shield blocks, or shield goes up.</t>
+          <t>Off-type hit.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>breaklayer</t>
+          <t>absorb</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>sawtooth</t>
+          <t>square</t>
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>760</v>
+        <v>300</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>80</v>
+        <v>1200</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>340</v>
+        <v>260</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>A layer flashes and breaks.</t>
+          <t>Same-type hit: the layer absorbs it.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>regrow</t>
+          <t>block</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>triangle</t>
+          <t>noise</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>120</v>
+        <v>1600</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>520</v>
+        <v>1600</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>300</v>
+        <v>90</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.16</v>
+        <v>0.3</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>The broken layer regrows at the back.</t>
+          <t>Shield blocks, or shield goes up.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>clash</t>
+          <t>breaklayer</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>sawtooth</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>240</v>
+        <v>760</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1500</v>
+        <v>340</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Death: the chevrons meet.</t>
+          <t>A layer flashes and breaks.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>speak</t>
+          <t>regrow</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>square</t>
+          <t>triangle</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>620</v>
+        <v>120</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>540</v>
+        <v>520</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>42</v>
+        <v>300</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0.09</v>
+        <v>0.16</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>0.12</v>
+        <v>0.4</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>One letter of dialogue appearing.</t>
+          <t>The broken layer regrows at the back.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>win</t>
+          <t>clash</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>square</t>
+          <t>noise</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>440</v>
+        <v>240</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>1320</v>
+        <v>240</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>620</v>
+        <v>1500</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.24</v>
+        <v>0.4</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>Victory.</t>
+          <t>Death: the chevrons meet.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>speak</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>540</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>One letter of dialogue appearing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>440</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Victory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
           <t>lose</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>sawtooth</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C20" s="8" t="n">
         <v>320</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D20" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E20" s="8" t="n">
         <v>950</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F20" s="8" t="n">
         <v>0.28</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G20" s="8" t="n">
         <v>0.6</v>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>Defeat.</t>
         </is>
@@ -2392,17 +2936,17 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>fury</t>
+          <t>anger</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>#ff4d3d</t>
+          <t>#e53859</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>#3a0509</t>
+          <t>#2a0810</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -2423,37 +2967,37 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>SADNESS</t>
+          <t>SURPRISE</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Sadness</t>
+          <t>Surprise</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>sorrow</t>
+          <t>surprise</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>#4a86ff</t>
+          <t>#724082</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>#061634</t>
+          <t>#170a1b</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>SAD</t>
+          <t>SUR</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Heavy, draining, persistent.</t>
+          <t>Sudden, disruptive, disorienting.</t>
         </is>
       </c>
       <c r="H6" s="8" t="n">
@@ -2464,37 +3008,37 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>JOY</t>
+          <t>DISGUST</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Joy</t>
+          <t>Disgust</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>euphoria</t>
+          <t>disgust</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>#ffc63d</t>
+          <t>#56a36a</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>#332305</t>
+          <t>#0c1f13</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>JOY</t>
+          <t>DIS</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Bright, volatile, energising.</t>
+          <t>Rejecting, corrosive, contemptuous.</t>
         </is>
       </c>
       <c r="H7" s="8" t="n">
@@ -2505,37 +3049,37 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>APATHY</t>
+          <t>JOY</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Apathy</t>
+          <t>Joy</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>apathy</t>
+          <t>joy</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>#8a7fa8</t>
+          <t>#fcc336</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>#1b1526</t>
+          <t>#2a1f06</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>JOY</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Blunt, numbing, absorbing.</t>
+          <t>Bright, volatile, energising.</t>
         </is>
       </c>
       <c r="H8" s="8" t="n">
@@ -2546,37 +3090,37 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>NOSTALGIA</t>
+          <t>SADNESS</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Nostalgia</t>
+          <t>Sadness</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>nostalgia</t>
+          <t>sadness</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>#ff5fae</t>
+          <t>#3d66c1</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>#330a1d</t>
+          <t>#0a1229</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>SAD</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Warm, distracting, sticky.</t>
+          <t>Heavy, draining, persistent.</t>
         </is>
       </c>
       <c r="H9" s="8" t="n">
@@ -2587,37 +3131,37 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>CALM</t>
+          <t>FEAR</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Calm</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>stoic</t>
+          <t>fear</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>#35d6b0</t>
+          <t>#929fa5</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>#052622</t>
+          <t>#1a1e20</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>CAL</t>
+          <t>FEA</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Steady, defensive, restorative.</t>
+          <t>Cold, freezing, evasive.</t>
         </is>
       </c>
       <c r="H10" s="8" t="n">
@@ -2663,7 +3207,7 @@
     <col width="17" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
     <col width="20" customWidth="1" min="25" max="25"/>
@@ -2794,7 +3338,7 @@
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>uses_per_battle</t>
+          <t>uses</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -2964,14 +3508,14 @@
           <t>planned</t>
         </is>
       </c>
-      <c r="U4" s="7" t="inlineStr">
-        <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="V4" s="7" t="inlineStr">
-        <is>
-          <t>planned</t>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="W4" s="7" t="inlineStr">
@@ -3116,10 +3660,10 @@
         <v>1</v>
       </c>
       <c r="U5" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W5" s="8" t="inlineStr"/>
       <c r="X5" s="8" t="n">
@@ -3231,10 +3775,10 @@
         <v>1</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W6" s="8" t="inlineStr"/>
       <c r="X6" s="8" t="n">
@@ -3346,10 +3890,10 @@
         <v>1</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W7" s="8" t="inlineStr"/>
       <c r="X7" s="8" t="n">
@@ -3457,10 +4001,10 @@
         <v>1</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V8" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W8" s="8" t="inlineStr"/>
       <c r="X8" s="8" t="n">
@@ -3572,10 +4116,10 @@
         <v>1</v>
       </c>
       <c r="U9" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W9" s="8" t="inlineStr"/>
       <c r="X9" s="8" t="n">
@@ -3687,10 +4231,10 @@
         <v>1</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W10" s="8" t="inlineStr"/>
       <c r="X10" s="8" t="n">
@@ -3802,10 +4346,10 @@
         <v>1</v>
       </c>
       <c r="U11" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W11" s="8" t="inlineStr"/>
       <c r="X11" s="8" t="n">
@@ -3913,10 +4457,10 @@
         <v>1</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W12" s="8" t="inlineStr"/>
       <c r="X12" s="8" t="n">
@@ -4509,12 +5053,12 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>SADNESS</t>
+          <t>SURPRISE</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>SADNESS</t>
+          <t>SURPRISE</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
@@ -4558,12 +5102,12 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>JOY</t>
+          <t>DISGUST</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>JOY</t>
+          <t>DISGUST</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
@@ -4607,12 +5151,12 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>APATHY</t>
+          <t>JOY</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>APATHY</t>
+          <t>JOY</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
@@ -4656,12 +5200,12 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>NOSTALGIA</t>
+          <t>SADNESS</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>NOSTALGIA</t>
+          <t>SADNESS</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
@@ -4705,12 +5249,12 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>CALM</t>
+          <t>FEAR</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>CALM</t>
+          <t>FEAR</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
@@ -4765,7 +5309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4776,13 +5320,15 @@
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4835,35 +5381,45 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
+          <t>line_cap</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>max_bonus_slots</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
           <t>ai_profile</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>init</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>start_shield</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>max_layers_override</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -4910,37 +5466,47 @@
           <t>LIVE</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="O4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="P4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="O4" s="7" t="inlineStr">
+      <c r="Q4" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
@@ -4977,23 +5543,29 @@
       <c r="H5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="8" t="inlineStr"/>
+      <c r="I5" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="J5" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" s="8" t="inlineStr"/>
+      <c r="L5" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="K5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="8" t="inlineStr"/>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8" t="inlineStr"/>
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>PLAYER</t>
         </is>
       </c>
-      <c r="N5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="8" t="inlineStr"/>
+      <c r="P5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -5024,33 +5596,39 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>ATK_ANGER|ATK_SADNESS|ATK_JOY|DEFEND|RECHARGE|HVY_ANGER</t>
+          <t>ATK_ANGER|ATK_SADNESS|ATK_JOY|DEFEND|RECHARGE|HVY_ANGER|HVY_SADNESS|HVY_JOY</t>
         </is>
       </c>
       <c r="H6" s="8" t="n">
         <v>-1</v>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>GREEDY_MAX_DAMAGE</t>
         </is>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="L6" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="K6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="8" t="inlineStr"/>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="M6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8" t="inlineStr"/>
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>ENEMY</t>
         </is>
       </c>
-      <c r="N6" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="8" t="inlineStr">
+      <c r="P6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
         <is>
           <t>AI reads the matchups sheet, so retuning it retunes the AI.</t>
         </is>
@@ -5058,7 +5636,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8728,7 +9306,7 @@
       </c>
       <c r="M5" s="8" t="inlineStr">
         <is>
-          <t>#8a7fa8</t>
+          <t>#929fa5</t>
         </is>
       </c>
       <c r="N5" s="8" t="n">

</xml_diff>